<commit_message>
Regression [Nightly 2026-06-26 02:26]: all — reports updated
</commit_message>
<xml_diff>
--- a/Test Execution Report/Daily Reports/BugReport_26-Jun-2026.xlsx
+++ b/Test Execution Report/Daily Reports/BugReport_26-Jun-2026.xlsx
@@ -3,8 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Daily Bug Report" sheetId="1" r:id="rId1"/>
-    <sheet name="Test Summary" sheetId="2" r:id="rId2"/>
+    <sheet name="Test Summary" sheetId="1" r:id="rId1"/>
+    <sheet name="Daily Bug Report" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
@@ -31,118 +31,17 @@
 </metadata>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
-  <si>
-    <t>Date</t>
-  </si>
-  <si>
-    <t>Module</t>
-  </si>
-  <si>
-    <t>TC ID</t>
-  </si>
-  <si>
-    <t>Test Case Name</t>
-  </si>
-  <si>
-    <t>Test Type</t>
-  </si>
-  <si>
-    <t>Priority</t>
-  </si>
-  <si>
-    <t>Status</t>
-  </si>
-  <si>
-    <t>Bug ID</t>
-  </si>
-  <si>
-    <t>Bug Title</t>
-  </si>
-  <si>
-    <t>Severity</t>
-  </si>
-  <si>
-    <t>Bug Priority</t>
-  </si>
-  <si>
-    <t>Environment</t>
-  </si>
-  <si>
-    <t>Browser</t>
-  </si>
-  <si>
-    <t>OS</t>
-  </si>
-  <si>
-    <t>Steps to Reproduce</t>
-  </si>
-  <si>
-    <t>Expected Result</t>
-  </si>
-  <si>
-    <t>Actual Result</t>
-  </si>
-  <si>
-    <t>Source Report</t>
-  </si>
-  <si>
-    <t>26-Jun-2026</t>
-  </si>
-  <si>
-    <t>Login</t>
-  </si>
-  <si>
-    <t>TC-LOGIN-001 to TC-LOGIN-020</t>
-  </si>
-  <si>
-    <t>All 20 Login test cases</t>
-  </si>
-  <si>
-    <t>Positive / Negative / Boundary / Security</t>
-  </si>
-  <si>
-    <t>Critical -- High -- Medium</t>
-  </si>
-  <si>
-    <t>ALL PASS (20/20)</t>
-  </si>
-  <si>
-    <t>--</t>
-  </si>
-  <si>
-    <t>No bugs found</t>
-  </si>
-  <si>
-    <t>http://customerportal.dev-ts.online</t>
-  </si>
-  <si>
-    <t>Chrome</t>
-  </si>
-  <si>
-    <t>Windows</t>
-  </si>
-  <si>
-    <t>All 20 tests pass</t>
-  </si>
-  <si>
-    <t>Test Execution Report\Feature Reports\Login.xlsx</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ap="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:op="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing" xmlns:comp="http://schemas.openxmlformats.org/drawingml/2006/compatibility" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:lc="http://schemas.openxmlformats.org/drawingml/2006/lockedCanvas" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xne="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mso="http://schemas.microsoft.com/office/2006/01/customui" xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:cppr="http://schemas.microsoft.com/office/2006/coverPageProps" xmlns:cdip="http://schemas.microsoft.com/office/2006/customDocumentInformationPanel" xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ntns="http://schemas.microsoft.com/office/2006/metadata/customXsn" xmlns:lp="http://schemas.microsoft.com/office/2006/metadata/longProperties" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" xmlns:msink="http://schemas.microsoft.com/ink/2010/main" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" xmlns:cdr14="http://schemas.microsoft.com/office/drawing/2010/chartDrawing" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns:pic14="http://schemas.microsoft.com/office/drawing/2010/picture" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:dsp="http://schemas.microsoft.com/office/drawing/2008/diagram" xmlns:mso14="http://schemas.microsoft.com/office/2009/07/customui" xmlns:dgm14="http://schemas.microsoft.com/office/drawing/2010/diagram" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:xr4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision4" xmlns:xr5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision5" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr7="http://schemas.microsoft.com/office/spreadsheetml/2016/revision7" xmlns:xr8="http://schemas.microsoft.com/office/spreadsheetml/2016/revision8" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr11="http://schemas.microsoft.com/office/spreadsheetml/2016/revision11" xmlns:xr12="http://schemas.microsoft.com/office/spreadsheetml/2016/revision12" xmlns:xr13="http://schemas.microsoft.com/office/spreadsheetml/2016/revision13" xmlns:xr14="http://schemas.microsoft.com/office/spreadsheetml/2016/revision14" xmlns:xr15="http://schemas.microsoft.com/office/spreadsheetml/2016/revision15" xmlns:x16="http://schemas.microsoft.com/office/spreadsheetml/2014/11/main" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:mo="http://schemas.microsoft.com/office/mac/office/2008/main" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:v="urn:schemas-microsoft-com:vml" mc:Ignorable="c14 cdr14 a14 pic14 x14 xdr14 x14ac dsp mso14 dgm14 x15 x12ac x15ac xr xr2 xr3 xr4 xr5 xr6 xr7 xr8 xr9 xr10 xr11 xr12 xr13 xr14 xr15 x15 x16 x16r2 mo mx mv o v" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
   <numFmts count="1">
     <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
   </numFmts>
   <fonts count="1">
     <font>
+      <sz val="12"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="12"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -167,18 +66,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultPivotStyle="PivotStyleMedium4" defaultTableStyle="TableStyleMedium9"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -499,133 +398,443 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R2"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" t="s">
-        <v>13</v>
-      </c>
-      <c r="O1" t="s">
-        <v>14</v>
-      </c>
-      <c r="P1" t="s">
-        <v>15</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>16</v>
-      </c>
-      <c r="R1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E2" t="s">
-        <v>22</v>
-      </c>
-      <c r="F2" t="s">
-        <v>23</v>
-      </c>
-      <c r="G2" t="s">
-        <v>24</v>
-      </c>
-      <c r="H2" t="s">
-        <v>25</v>
-      </c>
-      <c r="I2" t="s">
-        <v>26</v>
-      </c>
-      <c r="J2" t="s">
-        <v>25</v>
-      </c>
-      <c r="K2" t="s">
-        <v>25</v>
-      </c>
-      <c r="L2" t="s">
-        <v>27</v>
-      </c>
-      <c r="M2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N2" t="s">
-        <v>29</v>
-      </c>
-      <c r="O2" t="s">
-        <v>25</v>
-      </c>
-      <c r="P2" t="s">
-        <v>30</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>30</v>
-      </c>
-      <c r="R2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-  </sheetData>
+  <dimension ref="A1"/>
+  <sheetData/>
   <ignoredErrors>
-    <ignoredError sqref="A1" numberStoredAsText="true"/>
+    <ignoredError numberStoredAsText="1" sqref="A1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetData/>
+  <dimension ref="A1:R7"/>
+  <cols>
+    <col min="1" max="1" width="14.83203125" customWidth="1"/>
+    <col min="2" max="2" width="16.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="44.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="10.83203125" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" customWidth="1"/>
+    <col min="8" max="8" width="20.83203125" customWidth="1"/>
+    <col min="9" max="9" width="44.83203125" customWidth="1"/>
+    <col min="10" max="10" width="10.83203125" customWidth="1"/>
+    <col min="11" max="11" width="12.83203125" customWidth="1"/>
+    <col min="12" max="12" width="36.83203125" customWidth="1"/>
+    <col min="13" max="13" width="10.83203125" customWidth="1"/>
+    <col min="14" max="14" width="10.83203125" customWidth="1"/>
+    <col min="15" max="15" width="40.83203125" customWidth="1"/>
+    <col min="16" max="16" width="32.83203125" customWidth="1"/>
+    <col min="17" max="17" width="44.83203125" customWidth="1"/>
+    <col min="18" max="18" width="36.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Date</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Module</v>
+      </c>
+      <c r="C1" t="str">
+        <v>TC ID</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Test Case Name</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Test Type</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Priority</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Status</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Bug ID</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Bug Title</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Severity</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Bug Priority</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Environment</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Browser</v>
+      </c>
+      <c r="N1" t="str">
+        <v>OS</v>
+      </c>
+      <c r="O1" t="str">
+        <v>Steps to Reproduce</v>
+      </c>
+      <c r="P1" t="str">
+        <v>Expected Result</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>Actual Result</v>
+      </c>
+      <c r="R1" t="str">
+        <v>Source Report</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>26-Jun-2026</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Login</v>
+      </c>
+      <c r="C2" t="str">
+        <v>TC-LOGIN-001 to TC-LOGIN-020</v>
+      </c>
+      <c r="D2" t="str">
+        <v>All 20 Login test cases</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Positive / Negative / Boundary / Security</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Critical -- High -- Medium</v>
+      </c>
+      <c r="G2" t="str">
+        <v>ALL PASS (20/20)</v>
+      </c>
+      <c r="H2" t="str">
+        <v>--</v>
+      </c>
+      <c r="I2" t="str">
+        <v>No bugs found</v>
+      </c>
+      <c r="J2" t="str">
+        <v>--</v>
+      </c>
+      <c r="K2" t="str">
+        <v>--</v>
+      </c>
+      <c r="L2" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="M2" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="N2" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="O2" t="str">
+        <v>--</v>
+      </c>
+      <c r="P2" t="str">
+        <v>All 20 tests pass</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>All 20 tests pass</v>
+      </c>
+      <c r="R2" t="str">
+        <v>Test Execution Report\Feature Reports\Login.xlsx</v>
+      </c>
+    </row>
+    <row r="3" xml:space="preserve">
+      <c r="A3" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Dashboard Module</v>
+      </c>
+      <c r="C3" t="str">
+        <v>TC-DASH-002</v>
+      </c>
+      <c r="D3" t="str">
+        <v>TC-DASH-002 | All 4 stat cards visible with values</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Low</v>
+      </c>
+      <c r="G3" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="H3" t="str">
+        <v>BUG-DASHBOARD-MODULE-002</v>
+      </c>
+      <c r="I3" t="str">
+        <v>[FAIL] TC-DASH-002 | All 4 stat cards visible with values</v>
+      </c>
+      <c r="J3" t="str">
+        <v>Low</v>
+      </c>
+      <c r="K3" t="str">
+        <v>P3</v>
+      </c>
+      <c r="L3" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="M3" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="N3" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="O3" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to feature page
+2. Execute test steps
+3. Observe failure</v>
+      </c>
+      <c r="P3" t="str">
+        <v>Test should pass successfully</v>
+      </c>
+      <c r="Q3" t="str">
+        <v>Error: _x001b_[2mexpect(_x001b_[22m_x001b_[31mreceived_x001b_[39m_x001b_[2m)._x001b_[22mtoBeTruthy_x001b_[2m()_x001b_[22m  Received: _x001b_[31mfalse_x001b_[39m</v>
+      </c>
+      <c r="R3" t="str">
+        <v>Test Execution Report\Feature Reports\Dashboard Module.xlsx  |  Tracker: New — not yet in tracker</v>
+      </c>
+    </row>
+    <row r="4" xml:space="preserve">
+      <c r="A4" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Dashboard Module</v>
+      </c>
+      <c r="C4" t="str">
+        <v>TC-DASH-004</v>
+      </c>
+      <c r="D4" t="str">
+        <v>TC-DASH-004 | ANALYTICS tab shows analytics content</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Low</v>
+      </c>
+      <c r="G4" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="H4" t="str">
+        <v>BUG-DASHBOARD-MODULE-003</v>
+      </c>
+      <c r="I4" t="str">
+        <v>[FAIL] TC-DASH-004 | ANALYTICS tab shows analytics content</v>
+      </c>
+      <c r="J4" t="str">
+        <v>Low</v>
+      </c>
+      <c r="K4" t="str">
+        <v>P3</v>
+      </c>
+      <c r="L4" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="M4" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="N4" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="O4" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to feature page
+2. Execute test steps
+3. Observe failure</v>
+      </c>
+      <c r="P4" t="str">
+        <v>Test should pass successfully</v>
+      </c>
+      <c r="Q4" t="str">
+        <v>Error: _x001b_[2mexpect(_x001b_[22m_x001b_[31mreceived_x001b_[39m_x001b_[2m)._x001b_[22mtoBeTruthy_x001b_[2m()_x001b_[22m  Received: _x001b_[31mfalse_x001b_[39m</v>
+      </c>
+      <c r="R4" t="str">
+        <v>Test Execution Report\Feature Reports\Dashboard Module.xlsx  |  Tracker: New — not yet in tracker</v>
+      </c>
+    </row>
+    <row r="5" xml:space="preserve">
+      <c r="A5" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Dashboard Module</v>
+      </c>
+      <c r="C5" t="str">
+        <v>TC-DASH-005</v>
+      </c>
+      <c r="D5" t="str">
+        <v>TC-DASH-005 | Switch back to OVERVIEW from ANALYTICS</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Low</v>
+      </c>
+      <c r="G5" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="H5" t="str">
+        <v>BUG-DASHBOARD-MODULE-004</v>
+      </c>
+      <c r="I5" t="str">
+        <v>[FAIL] TC-DASH-005 | Switch back to OVERVIEW from ANALYTICS</v>
+      </c>
+      <c r="J5" t="str">
+        <v>Low</v>
+      </c>
+      <c r="K5" t="str">
+        <v>P3</v>
+      </c>
+      <c r="L5" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="M5" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="N5" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="O5" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to feature page
+2. Execute test steps
+3. Observe failure</v>
+      </c>
+      <c r="P5" t="str">
+        <v>Test should pass successfully</v>
+      </c>
+      <c r="Q5" t="str">
+        <v>Error: _x001b_[2mexpect(_x001b_[22m_x001b_[31mreceived_x001b_[39m_x001b_[2m)._x001b_[22mtoBeTruthy_x001b_[2m()_x001b_[22m  Received: _x001b_[31mfalse_x001b_[39m</v>
+      </c>
+      <c r="R5" t="str">
+        <v>Test Execution Report\Feature Reports\Dashboard Module.xlsx  |  Tracker: New — not yet in tracker</v>
+      </c>
+    </row>
+    <row r="6" xml:space="preserve">
+      <c r="A6" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Dashboard Module</v>
+      </c>
+      <c r="C6" t="str">
+        <v>TC-DASH-011</v>
+      </c>
+      <c r="D6" t="str">
+        <v>TC-DASH-011 | All sidebar navigation links present</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Low</v>
+      </c>
+      <c r="G6" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="H6" t="str">
+        <v>BUG-DASHBOARD-MODULE-005</v>
+      </c>
+      <c r="I6" t="str">
+        <v>[FAIL] TC-DASH-011 | All sidebar navigation links present</v>
+      </c>
+      <c r="J6" t="str">
+        <v>Low</v>
+      </c>
+      <c r="K6" t="str">
+        <v>P3</v>
+      </c>
+      <c r="L6" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="M6" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="N6" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="O6" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to feature page
+2. Execute test steps
+3. Observe failure</v>
+      </c>
+      <c r="P6" t="str">
+        <v>Test should pass successfully</v>
+      </c>
+      <c r="Q6" t="str">
+        <v>Error: _x001b_[2mexpect(_x001b_[22m_x001b_[31mlocator_x001b_[39m_x001b_[2m)._x001b_[22mtoBeVisible_x001b_[2m(_x001b_[22m_x001b_[2m)_x001b_[22m failed  Locator:  locator('a[href="/Ticket/Index"]').first() Expected: visible Received: hidden Timeout:  5000ms  Cal</v>
+      </c>
+      <c r="R6" t="str">
+        <v>Test Execution Report\Feature Reports\Dashboard Module.xlsx  |  Tracker: New — not yet in tracker</v>
+      </c>
+    </row>
+    <row r="7" xml:space="preserve">
+      <c r="A7" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Dashboard Module</v>
+      </c>
+      <c r="C7" t="str">
+        <v>TC-DASH-012</v>
+      </c>
+      <c r="D7" t="str">
+        <v>TC-DASH-012 | Action Queue badge shows ticket count</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Low</v>
+      </c>
+      <c r="G7" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="H7" t="str">
+        <v>BUG-DASHBOARD-MODULE-006</v>
+      </c>
+      <c r="I7" t="str">
+        <v>[FAIL] TC-DASH-012 | Action Queue badge shows ticket count</v>
+      </c>
+      <c r="J7" t="str">
+        <v>Low</v>
+      </c>
+      <c r="K7" t="str">
+        <v>P3</v>
+      </c>
+      <c r="L7" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="M7" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="N7" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="O7" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to feature page
+2. Execute test steps
+3. Observe failure</v>
+      </c>
+      <c r="P7" t="str">
+        <v>Test should pass successfully</v>
+      </c>
+      <c r="Q7" t="str">
+        <v>Error: _x001b_[2mexpect(_x001b_[22m_x001b_[31mreceived_x001b_[39m_x001b_[2m)._x001b_[22mtoBeTruthy_x001b_[2m()_x001b_[22m  Received: _x001b_[31mfalse_x001b_[39m</v>
+      </c>
+      <c r="R7" t="str">
+        <v>Test Execution Report\Feature Reports\Dashboard Module.xlsx  |  Tracker: New — not yet in tracker</v>
+      </c>
+    </row>
+  </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:R7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
CI Reports [2026-06-26 08:04]: All — Excel reports updated
</commit_message>
<xml_diff>
--- a/Test Execution Report/Daily Reports/BugReport_26-Jun-2026.xlsx
+++ b/Test Execution Report/Daily Reports/BugReport_26-Jun-2026.xlsx
@@ -408,7 +408,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R7"/>
+  <dimension ref="A1:T15"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -485,6 +485,12 @@
       <c r="R1" t="str">
         <v>Source Report</v>
       </c>
+      <c r="S1" t="str">
+        <v>Feature</v>
+      </c>
+      <c r="T1" t="str">
+        <v>Layer</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -832,9 +838,481 @@
         <v>Test Execution Report\Feature Reports\Dashboard Module.xlsx  |  Tracker: New — not yet in tracker</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="C8" t="str">
+        <v>TC-TICKET-001</v>
+      </c>
+      <c r="D8" t="str">
+        <v>TC-TICKET-001 | Create Ticket page loads with all required fields</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Critical</v>
+      </c>
+      <c r="G8" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="H8" t="str">
+        <v>BUG-CREATETICKET-007</v>
+      </c>
+      <c r="I8" t="str">
+        <v>[FAIL] TC-TICKET-001 | Create Ticket page loads with all required fields</v>
+      </c>
+      <c r="J8" t="str">
+        <v>Critical</v>
+      </c>
+      <c r="K8" t="str">
+        <v>P1</v>
+      </c>
+      <c r="L8" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="M8" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="N8" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="O8" t="str">
+        <v>See spec: tests/createticket.spec.js  TC: TC-TICKET-001</v>
+      </c>
+      <c r="P8" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="Q8" t="str">
+        <v>Error: expect(page).toHaveTitle(expected) failed Expected pattern: /Create Ticket/i Received string: "Sign In" Timeout: 5000ms Call log: - Expect "toHaveTitle" with timeout 5000ms 14 × unexpected value "Sign In"</v>
+      </c>
+      <c r="R8" t="str">
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
+      </c>
+      <c r="S8" t="str">
+        <v>CreateTicket</v>
+      </c>
+      <c r="T8" t="str">
+        <v>Auto</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="C9" t="str">
+        <v>TC-TICKET-005</v>
+      </c>
+      <c r="D9" t="str">
+        <v>TC-TICKET-005 | All Ticket Type chips are visible</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Low</v>
+      </c>
+      <c r="G9" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="H9" t="str">
+        <v>BUG-CREATETICKET-008</v>
+      </c>
+      <c r="I9" t="str">
+        <v>[FAIL] TC-TICKET-005 | All Ticket Type chips are visible</v>
+      </c>
+      <c r="J9" t="str">
+        <v>Low</v>
+      </c>
+      <c r="K9" t="str">
+        <v>P3</v>
+      </c>
+      <c r="L9" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="M9" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="N9" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="O9" t="str">
+        <v>See spec: tests/createticket.spec.js  TC: TC-TICKET-005</v>
+      </c>
+      <c r="P9" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="Q9" t="str">
+        <v>Error: expect(locator).toBeVisible() failed Locator: locator('#typeChips .ct-type-chip').filter({ hasText: 'New' }).first() Expected: visible Timeout: 5000ms Error: element(s) not found Call log: - Expect "toBeVisible" with timeout 5000ms - waiting for locator('#typeChips .ct-type-chip').filter({ ha</v>
+      </c>
+      <c r="R9" t="str">
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
+      </c>
+      <c r="S9" t="str">
+        <v>CreateTicket</v>
+      </c>
+      <c r="T9" t="str">
+        <v>Auto</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="C10" t="str">
+        <v>TC-DASH-003</v>
+      </c>
+      <c r="D10" t="str">
+        <v>TC-DASH-003 | OVERVIEW and ANALYTICS buttons visible</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Low</v>
+      </c>
+      <c r="G10" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="H10" t="str">
+        <v>BUG-CREATETICKET-009</v>
+      </c>
+      <c r="I10" t="str">
+        <v>[FAIL] TC-DASH-003 | OVERVIEW and ANALYTICS buttons visible</v>
+      </c>
+      <c r="J10" t="str">
+        <v>Low</v>
+      </c>
+      <c r="K10" t="str">
+        <v>P3</v>
+      </c>
+      <c r="L10" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="M10" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="N10" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="O10" t="str">
+        <v>See spec: tests/createticket.spec.js  TC: TC-DASH-003</v>
+      </c>
+      <c r="P10" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="Q10" t="str">
+        <v>Error: expect(locator).toBeVisible() failed Locator: locator('#btnOverview') Expected: visible Timeout: 5000ms Error: element(s) not found Call log: - Expect "toBeVisible" with timeout 5000ms - waiting for locator('#btnOverview')</v>
+      </c>
+      <c r="R10" t="str">
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
+      </c>
+      <c r="S10" t="str">
+        <v>CreateTicket</v>
+      </c>
+      <c r="T10" t="str">
+        <v>Auto</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="C11" t="str">
+        <v>TC-DASH-009</v>
+      </c>
+      <c r="D11" t="str">
+        <v>TC-DASH-009 | Active Tickets table with correct columns</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F11" t="str">
+        <v>Low</v>
+      </c>
+      <c r="G11" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="H11" t="str">
+        <v>BUG-CREATETICKET-010</v>
+      </c>
+      <c r="I11" t="str">
+        <v>[FAIL] TC-DASH-009 | Active Tickets table with correct columns</v>
+      </c>
+      <c r="J11" t="str">
+        <v>Low</v>
+      </c>
+      <c r="K11" t="str">
+        <v>P3</v>
+      </c>
+      <c r="L11" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="M11" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="N11" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="O11" t="str">
+        <v>See spec: tests/createticket.spec.js  TC: TC-DASH-009</v>
+      </c>
+      <c r="P11" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="Q11" t="str">
+        <v>Error: expect(locator).toBeVisible() failed Locator: locator('table').first() Expected: visible Timeout: 5000ms Error: element(s) not found Call log: - Expect "toBeVisible" with timeout 5000ms - waiting for locator('table').first()</v>
+      </c>
+      <c r="R11" t="str">
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
+      </c>
+      <c r="S11" t="str">
+        <v>CreateTicket</v>
+      </c>
+      <c r="T11" t="str">
+        <v>Auto</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="C12" t="str">
+        <v>TC-DASH-013</v>
+      </c>
+      <c r="D12" t="str">
+        <v>TC-DASH-013 | Search box accepts input</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F12" t="str">
+        <v>Low</v>
+      </c>
+      <c r="G12" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="H12" t="str">
+        <v>BUG-CREATETICKET-011</v>
+      </c>
+      <c r="I12" t="str">
+        <v>[FAIL] TC-DASH-013 | Search box accepts input</v>
+      </c>
+      <c r="J12" t="str">
+        <v>Low</v>
+      </c>
+      <c r="K12" t="str">
+        <v>P3</v>
+      </c>
+      <c r="L12" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="M12" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="N12" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="O12" t="str">
+        <v>See spec: tests/createticket.spec.js  TC: TC-DASH-013</v>
+      </c>
+      <c r="P12" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="Q12" t="str">
+        <v>Error: expect(locator).toBeVisible() failed Locator: locator('input[placeholder="Search"]').first() Expected: visible Timeout: 5000ms Error: element(s) not found Call log: - Expect "toBeVisible" with timeout 5000ms - waiting for locator('input[placeholder="Search"]').first()</v>
+      </c>
+      <c r="R12" t="str">
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
+      </c>
+      <c r="S12" t="str">
+        <v>CreateTicket</v>
+      </c>
+      <c r="T12" t="str">
+        <v>Auto</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="C13" t="str">
+        <v>CreateTicket-passed-26 Jun 2026</v>
+      </c>
+      <c r="D13" t="str">
+        <v>25 TCs passed — CreateTicket (FAILs above)</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Mixed</v>
+      </c>
+      <c r="F13" t="str">
+        <v>Mixed</v>
+      </c>
+      <c r="G13" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="H13" t="str">
+        <v>—</v>
+      </c>
+      <c r="I13" t="str">
+        <v>25/55 TCs passed</v>
+      </c>
+      <c r="J13" t="str">
+        <v>—</v>
+      </c>
+      <c r="K13" t="str">
+        <v>—</v>
+      </c>
+      <c r="L13" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="M13" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="N13" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="O13" t="str">
+        <v>Playwright run: tests/createticket.spec.js</v>
+      </c>
+      <c r="P13" t="str">
+        <v>Assertions pass</v>
+      </c>
+      <c r="Q13" t="str">
+        <v>25/55 PASS | 10 FAILs logged</v>
+      </c>
+      <c r="R13" t="str">
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
+      </c>
+      <c r="S13" t="str">
+        <v>CreateTicket</v>
+      </c>
+      <c r="T13" t="str">
+        <v>Mixed</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Dashboard-passed-26 Jun 2026</v>
+      </c>
+      <c r="D14" t="str">
+        <v>25 TCs passed — Dashboard (FAILs above)</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Mixed</v>
+      </c>
+      <c r="F14" t="str">
+        <v>Mixed</v>
+      </c>
+      <c r="G14" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="H14" t="str">
+        <v>—</v>
+      </c>
+      <c r="I14" t="str">
+        <v>25/55 TCs passed</v>
+      </c>
+      <c r="J14" t="str">
+        <v>—</v>
+      </c>
+      <c r="K14" t="str">
+        <v>—</v>
+      </c>
+      <c r="L14" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="M14" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="N14" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="O14" t="str">
+        <v>Playwright run: tests/dashboard.spec.js</v>
+      </c>
+      <c r="P14" t="str">
+        <v>Assertions pass</v>
+      </c>
+      <c r="Q14" t="str">
+        <v>25/55 PASS | 10 FAILs logged</v>
+      </c>
+      <c r="R14" t="str">
+        <v>Test Execution Report\Feature Reports\Dashboard.xlsx</v>
+      </c>
+      <c r="S14" t="str">
+        <v>Dashboard</v>
+      </c>
+      <c r="T14" t="str">
+        <v>Mixed</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Login-passed-26 Jun 2026</v>
+      </c>
+      <c r="D15" t="str">
+        <v>25 TCs passed — Login (FAILs above)</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Mixed</v>
+      </c>
+      <c r="F15" t="str">
+        <v>Mixed</v>
+      </c>
+      <c r="G15" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="H15" t="str">
+        <v>—</v>
+      </c>
+      <c r="I15" t="str">
+        <v>25/55 TCs passed</v>
+      </c>
+      <c r="J15" t="str">
+        <v>—</v>
+      </c>
+      <c r="K15" t="str">
+        <v>—</v>
+      </c>
+      <c r="L15" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="M15" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="N15" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="O15" t="str">
+        <v>Playwright run: tests/login.spec.js</v>
+      </c>
+      <c r="P15" t="str">
+        <v>Assertions pass</v>
+      </c>
+      <c r="Q15" t="str">
+        <v>25/55 PASS | 10 FAILs logged</v>
+      </c>
+      <c r="R15" t="str">
+        <v>Test Execution Report\Feature Reports\Login.xlsx</v>
+      </c>
+      <c r="S15" t="str">
+        <v>Login</v>
+      </c>
+      <c r="T15" t="str">
+        <v>Mixed</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:R7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:T15"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
CI Reports [2026-06-26 09:12]: All — Excel reports updated
</commit_message>
<xml_diff>
--- a/Test Execution Report/Daily Reports/BugReport_26-Jun-2026.xlsx
+++ b/Test Execution Report/Daily Reports/BugReport_26-Jun-2026.xlsx
@@ -408,26 +408,27 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T15"/>
+  <dimension ref="A1:T35"/>
   <cols>
-    <col min="1" max="1" width="14.83203125" customWidth="1"/>
-    <col min="2" max="2" width="16.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="1" max="1" width="13.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="22.83203125" customWidth="1"/>
     <col min="4" max="4" width="44.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" customWidth="1"/>
     <col min="6" max="6" width="10.83203125" customWidth="1"/>
-    <col min="7" max="7" width="12.83203125" customWidth="1"/>
-    <col min="8" max="8" width="20.83203125" customWidth="1"/>
-    <col min="9" max="9" width="44.83203125" customWidth="1"/>
-    <col min="10" max="10" width="10.83203125" customWidth="1"/>
-    <col min="11" max="11" width="12.83203125" customWidth="1"/>
-    <col min="12" max="12" width="36.83203125" customWidth="1"/>
-    <col min="13" max="13" width="10.83203125" customWidth="1"/>
-    <col min="14" max="14" width="10.83203125" customWidth="1"/>
-    <col min="15" max="15" width="40.83203125" customWidth="1"/>
-    <col min="16" max="16" width="32.83203125" customWidth="1"/>
-    <col min="17" max="17" width="44.83203125" customWidth="1"/>
-    <col min="18" max="18" width="36.83203125" customWidth="1"/>
+    <col min="7" max="7" width="10.83203125" customWidth="1"/>
+    <col min="8" max="8" width="8.83203125" customWidth="1"/>
+    <col min="9" max="9" width="20.83203125" customWidth="1"/>
+    <col min="10" max="10" width="46.83203125" customWidth="1"/>
+    <col min="11" max="11" width="10.83203125" customWidth="1"/>
+    <col min="12" max="12" width="10.83203125" customWidth="1"/>
+    <col min="13" max="13" width="36.83203125" customWidth="1"/>
+    <col min="14" max="14" width="9.83203125" customWidth="1"/>
+    <col min="15" max="15" width="9.83203125" customWidth="1"/>
+    <col min="16" max="16" width="44.83203125" customWidth="1"/>
+    <col min="17" max="17" width="36.83203125" customWidth="1"/>
+    <col min="18" max="18" width="50.83203125" customWidth="1"/>
+    <col min="19" max="19" width="40.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -435,7 +436,7 @@
         <v>Date</v>
       </c>
       <c r="B1" t="str">
-        <v>Module</v>
+        <v>Feature</v>
       </c>
       <c r="C1" t="str">
         <v>TC ID</v>
@@ -447,58 +448,55 @@
         <v>Test Type</v>
       </c>
       <c r="F1" t="str">
+        <v>Layer</v>
+      </c>
+      <c r="G1" t="str">
         <v>Priority</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>Status</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>Bug ID</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>Bug Title</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>Severity</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>Bug Priority</v>
       </c>
-      <c r="L1" t="str">
+      <c r="M1" t="str">
         <v>Environment</v>
       </c>
-      <c r="M1" t="str">
+      <c r="N1" t="str">
         <v>Browser</v>
       </c>
-      <c r="N1" t="str">
+      <c r="O1" t="str">
         <v>OS</v>
       </c>
-      <c r="O1" t="str">
+      <c r="P1" t="str">
         <v>Steps to Reproduce</v>
       </c>
-      <c r="P1" t="str">
+      <c r="Q1" t="str">
         <v>Expected Result</v>
       </c>
-      <c r="Q1" t="str">
+      <c r="R1" t="str">
         <v>Actual Result</v>
       </c>
-      <c r="R1" t="str">
+      <c r="S1" t="str">
         <v>Source Report</v>
       </c>
-      <c r="S1" t="str">
-        <v>Feature</v>
-      </c>
       <c r="T1" t="str">
-        <v>Layer</v>
+        <v>Module</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
         <v>26-Jun-2026</v>
       </c>
-      <c r="B2" t="str">
-        <v>Login</v>
-      </c>
       <c r="C2" t="str">
         <v>TC-LOGIN-001 to TC-LOGIN-020</v>
       </c>
@@ -508,53 +506,53 @@
       <c r="E2" t="str">
         <v>Positive / Negative / Boundary / Security</v>
       </c>
-      <c r="F2" t="str">
+      <c r="G2" t="str">
         <v>Critical -- High -- Medium</v>
       </c>
-      <c r="G2" t="str">
+      <c r="H2" t="str">
         <v>ALL PASS (20/20)</v>
       </c>
-      <c r="H2" t="str">
+      <c r="I2" t="str">
         <v>--</v>
       </c>
-      <c r="I2" t="str">
+      <c r="J2" t="str">
         <v>No bugs found</v>
-      </c>
-      <c r="J2" t="str">
-        <v>--</v>
       </c>
       <c r="K2" t="str">
         <v>--</v>
       </c>
       <c r="L2" t="str">
-        <v>http://customerportal.dev-ts.online</v>
+        <v>--</v>
       </c>
       <c r="M2" t="str">
-        <v>Chrome</v>
+        <v>http://customerportal.dev-ts.online</v>
       </c>
       <c r="N2" t="str">
-        <v>Windows</v>
+        <v>Chrome</v>
       </c>
       <c r="O2" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P2" t="str">
         <v>--</v>
-      </c>
-      <c r="P2" t="str">
-        <v>All 20 tests pass</v>
       </c>
       <c r="Q2" t="str">
         <v>All 20 tests pass</v>
       </c>
       <c r="R2" t="str">
+        <v>All 20 tests pass</v>
+      </c>
+      <c r="S2" t="str">
         <v>Test Execution Report\Feature Reports\Login.xlsx</v>
+      </c>
+      <c r="T2" t="str">
+        <v>Login</v>
       </c>
     </row>
     <row r="3" xml:space="preserve">
       <c r="A3" t="str">
         <v>26 Jun 2026</v>
       </c>
-      <c r="B3" t="str">
-        <v>Dashboard Module</v>
-      </c>
       <c r="C3" t="str">
         <v>TC-DASH-002</v>
       </c>
@@ -564,55 +562,55 @@
       <c r="E3" t="str">
         <v>Positive</v>
       </c>
-      <c r="F3" t="str">
-        <v>Low</v>
-      </c>
       <c r="G3" t="str">
-        <v>FAIL</v>
+        <v>Low</v>
       </c>
       <c r="H3" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I3" t="str">
         <v>BUG-DASHBOARD-MODULE-002</v>
       </c>
-      <c r="I3" t="str">
+      <c r="J3" t="str">
         <v>[FAIL] TC-DASH-002 | All 4 stat cards visible with values</v>
       </c>
-      <c r="J3" t="str">
-        <v>Low</v>
-      </c>
       <c r="K3" t="str">
-        <v>P3</v>
+        <v>Low</v>
       </c>
       <c r="L3" t="str">
-        <v>http://customerportal.dev-ts.online</v>
+        <v>P3</v>
       </c>
       <c r="M3" t="str">
-        <v>Chrome</v>
+        <v>http://customerportal.dev-ts.online</v>
       </c>
       <c r="N3" t="str">
-        <v>Windows</v>
-      </c>
-      <c r="O3" t="str" xml:space="preserve">
+        <v>Chrome</v>
+      </c>
+      <c r="O3" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P3" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Navigate to feature page
 2. Execute test steps
 3. Observe failure</v>
       </c>
-      <c r="P3" t="str">
+      <c r="Q3" t="str">
         <v>Test should pass successfully</v>
       </c>
-      <c r="Q3" t="str">
+      <c r="R3" t="str">
         <v>Error: _x001b_[2mexpect(_x001b_[22m_x001b_[31mreceived_x001b_[39m_x001b_[2m)._x001b_[22mtoBeTruthy_x001b_[2m()_x001b_[22m  Received: _x001b_[31mfalse_x001b_[39m</v>
       </c>
-      <c r="R3" t="str">
+      <c r="S3" t="str">
         <v>Test Execution Report\Feature Reports\Dashboard Module.xlsx  |  Tracker: New — not yet in tracker</v>
+      </c>
+      <c r="T3" t="str">
+        <v>Dashboard Module</v>
       </c>
     </row>
     <row r="4" xml:space="preserve">
       <c r="A4" t="str">
         <v>26 Jun 2026</v>
       </c>
-      <c r="B4" t="str">
-        <v>Dashboard Module</v>
-      </c>
       <c r="C4" t="str">
         <v>TC-DASH-004</v>
       </c>
@@ -622,55 +620,55 @@
       <c r="E4" t="str">
         <v>Positive</v>
       </c>
-      <c r="F4" t="str">
-        <v>Low</v>
-      </c>
       <c r="G4" t="str">
-        <v>FAIL</v>
+        <v>Low</v>
       </c>
       <c r="H4" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I4" t="str">
         <v>BUG-DASHBOARD-MODULE-003</v>
       </c>
-      <c r="I4" t="str">
+      <c r="J4" t="str">
         <v>[FAIL] TC-DASH-004 | ANALYTICS tab shows analytics content</v>
       </c>
-      <c r="J4" t="str">
-        <v>Low</v>
-      </c>
       <c r="K4" t="str">
-        <v>P3</v>
+        <v>Low</v>
       </c>
       <c r="L4" t="str">
-        <v>http://customerportal.dev-ts.online</v>
+        <v>P3</v>
       </c>
       <c r="M4" t="str">
-        <v>Chrome</v>
+        <v>http://customerportal.dev-ts.online</v>
       </c>
       <c r="N4" t="str">
-        <v>Windows</v>
-      </c>
-      <c r="O4" t="str" xml:space="preserve">
+        <v>Chrome</v>
+      </c>
+      <c r="O4" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P4" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Navigate to feature page
 2. Execute test steps
 3. Observe failure</v>
       </c>
-      <c r="P4" t="str">
+      <c r="Q4" t="str">
         <v>Test should pass successfully</v>
       </c>
-      <c r="Q4" t="str">
+      <c r="R4" t="str">
         <v>Error: _x001b_[2mexpect(_x001b_[22m_x001b_[31mreceived_x001b_[39m_x001b_[2m)._x001b_[22mtoBeTruthy_x001b_[2m()_x001b_[22m  Received: _x001b_[31mfalse_x001b_[39m</v>
       </c>
-      <c r="R4" t="str">
+      <c r="S4" t="str">
         <v>Test Execution Report\Feature Reports\Dashboard Module.xlsx  |  Tracker: New — not yet in tracker</v>
+      </c>
+      <c r="T4" t="str">
+        <v>Dashboard Module</v>
       </c>
     </row>
     <row r="5" xml:space="preserve">
       <c r="A5" t="str">
         <v>26 Jun 2026</v>
       </c>
-      <c r="B5" t="str">
-        <v>Dashboard Module</v>
-      </c>
       <c r="C5" t="str">
         <v>TC-DASH-005</v>
       </c>
@@ -680,55 +678,55 @@
       <c r="E5" t="str">
         <v>Positive</v>
       </c>
-      <c r="F5" t="str">
-        <v>Low</v>
-      </c>
       <c r="G5" t="str">
-        <v>FAIL</v>
+        <v>Low</v>
       </c>
       <c r="H5" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I5" t="str">
         <v>BUG-DASHBOARD-MODULE-004</v>
       </c>
-      <c r="I5" t="str">
+      <c r="J5" t="str">
         <v>[FAIL] TC-DASH-005 | Switch back to OVERVIEW from ANALYTICS</v>
       </c>
-      <c r="J5" t="str">
-        <v>Low</v>
-      </c>
       <c r="K5" t="str">
-        <v>P3</v>
+        <v>Low</v>
       </c>
       <c r="L5" t="str">
-        <v>http://customerportal.dev-ts.online</v>
+        <v>P3</v>
       </c>
       <c r="M5" t="str">
-        <v>Chrome</v>
+        <v>http://customerportal.dev-ts.online</v>
       </c>
       <c r="N5" t="str">
-        <v>Windows</v>
-      </c>
-      <c r="O5" t="str" xml:space="preserve">
+        <v>Chrome</v>
+      </c>
+      <c r="O5" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P5" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Navigate to feature page
 2. Execute test steps
 3. Observe failure</v>
       </c>
-      <c r="P5" t="str">
+      <c r="Q5" t="str">
         <v>Test should pass successfully</v>
       </c>
-      <c r="Q5" t="str">
+      <c r="R5" t="str">
         <v>Error: _x001b_[2mexpect(_x001b_[22m_x001b_[31mreceived_x001b_[39m_x001b_[2m)._x001b_[22mtoBeTruthy_x001b_[2m()_x001b_[22m  Received: _x001b_[31mfalse_x001b_[39m</v>
       </c>
-      <c r="R5" t="str">
+      <c r="S5" t="str">
         <v>Test Execution Report\Feature Reports\Dashboard Module.xlsx  |  Tracker: New — not yet in tracker</v>
+      </c>
+      <c r="T5" t="str">
+        <v>Dashboard Module</v>
       </c>
     </row>
     <row r="6" xml:space="preserve">
       <c r="A6" t="str">
         <v>26 Jun 2026</v>
       </c>
-      <c r="B6" t="str">
-        <v>Dashboard Module</v>
-      </c>
       <c r="C6" t="str">
         <v>TC-DASH-011</v>
       </c>
@@ -738,55 +736,55 @@
       <c r="E6" t="str">
         <v>Positive</v>
       </c>
-      <c r="F6" t="str">
-        <v>Low</v>
-      </c>
       <c r="G6" t="str">
-        <v>FAIL</v>
+        <v>Low</v>
       </c>
       <c r="H6" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I6" t="str">
         <v>BUG-DASHBOARD-MODULE-005</v>
       </c>
-      <c r="I6" t="str">
+      <c r="J6" t="str">
         <v>[FAIL] TC-DASH-011 | All sidebar navigation links present</v>
       </c>
-      <c r="J6" t="str">
-        <v>Low</v>
-      </c>
       <c r="K6" t="str">
-        <v>P3</v>
+        <v>Low</v>
       </c>
       <c r="L6" t="str">
-        <v>http://customerportal.dev-ts.online</v>
+        <v>P3</v>
       </c>
       <c r="M6" t="str">
-        <v>Chrome</v>
+        <v>http://customerportal.dev-ts.online</v>
       </c>
       <c r="N6" t="str">
-        <v>Windows</v>
-      </c>
-      <c r="O6" t="str" xml:space="preserve">
+        <v>Chrome</v>
+      </c>
+      <c r="O6" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P6" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Navigate to feature page
 2. Execute test steps
 3. Observe failure</v>
       </c>
-      <c r="P6" t="str">
+      <c r="Q6" t="str">
         <v>Test should pass successfully</v>
       </c>
-      <c r="Q6" t="str">
+      <c r="R6" t="str">
         <v>Error: _x001b_[2mexpect(_x001b_[22m_x001b_[31mlocator_x001b_[39m_x001b_[2m)._x001b_[22mtoBeVisible_x001b_[2m(_x001b_[22m_x001b_[2m)_x001b_[22m failed  Locator:  locator('a[href="/Ticket/Index"]').first() Expected: visible Received: hidden Timeout:  5000ms  Cal</v>
       </c>
-      <c r="R6" t="str">
+      <c r="S6" t="str">
         <v>Test Execution Report\Feature Reports\Dashboard Module.xlsx  |  Tracker: New — not yet in tracker</v>
+      </c>
+      <c r="T6" t="str">
+        <v>Dashboard Module</v>
       </c>
     </row>
     <row r="7" xml:space="preserve">
       <c r="A7" t="str">
         <v>26 Jun 2026</v>
       </c>
-      <c r="B7" t="str">
-        <v>Dashboard Module</v>
-      </c>
       <c r="C7" t="str">
         <v>TC-DASH-012</v>
       </c>
@@ -796,52 +794,58 @@
       <c r="E7" t="str">
         <v>Positive</v>
       </c>
-      <c r="F7" t="str">
-        <v>Low</v>
-      </c>
       <c r="G7" t="str">
-        <v>FAIL</v>
+        <v>Low</v>
       </c>
       <c r="H7" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I7" t="str">
         <v>BUG-DASHBOARD-MODULE-006</v>
       </c>
-      <c r="I7" t="str">
+      <c r="J7" t="str">
         <v>[FAIL] TC-DASH-012 | Action Queue badge shows ticket count</v>
       </c>
-      <c r="J7" t="str">
-        <v>Low</v>
-      </c>
       <c r="K7" t="str">
-        <v>P3</v>
+        <v>Low</v>
       </c>
       <c r="L7" t="str">
-        <v>http://customerportal.dev-ts.online</v>
+        <v>P3</v>
       </c>
       <c r="M7" t="str">
-        <v>Chrome</v>
+        <v>http://customerportal.dev-ts.online</v>
       </c>
       <c r="N7" t="str">
-        <v>Windows</v>
-      </c>
-      <c r="O7" t="str" xml:space="preserve">
+        <v>Chrome</v>
+      </c>
+      <c r="O7" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P7" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Navigate to feature page
 2. Execute test steps
 3. Observe failure</v>
       </c>
-      <c r="P7" t="str">
+      <c r="Q7" t="str">
         <v>Test should pass successfully</v>
       </c>
-      <c r="Q7" t="str">
+      <c r="R7" t="str">
         <v>Error: _x001b_[2mexpect(_x001b_[22m_x001b_[31mreceived_x001b_[39m_x001b_[2m)._x001b_[22mtoBeTruthy_x001b_[2m()_x001b_[22m  Received: _x001b_[31mfalse_x001b_[39m</v>
       </c>
-      <c r="R7" t="str">
+      <c r="S7" t="str">
         <v>Test Execution Report\Feature Reports\Dashboard Module.xlsx  |  Tracker: New — not yet in tracker</v>
+      </c>
+      <c r="T7" t="str">
+        <v>Dashboard Module</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
         <v>26 Jun 2026</v>
       </c>
+      <c r="B8" t="str">
+        <v>CreateTicket</v>
+      </c>
       <c r="C8" t="str">
         <v>TC-TICKET-001</v>
       </c>
@@ -852,55 +856,55 @@
         <v>Positive</v>
       </c>
       <c r="F8" t="str">
+        <v>Auto</v>
+      </c>
+      <c r="G8" t="str">
         <v>Critical</v>
       </c>
-      <c r="G8" t="str">
-        <v>FAIL</v>
-      </c>
       <c r="H8" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I8" t="str">
         <v>BUG-CREATETICKET-007</v>
       </c>
-      <c r="I8" t="str">
+      <c r="J8" t="str">
         <v>[FAIL] TC-TICKET-001 | Create Ticket page loads with all required fields</v>
       </c>
-      <c r="J8" t="str">
+      <c r="K8" t="str">
         <v>Critical</v>
       </c>
-      <c r="K8" t="str">
+      <c r="L8" t="str">
         <v>P1</v>
       </c>
-      <c r="L8" t="str">
-        <v>http://customerportal.dev-ts.online</v>
-      </c>
       <c r="M8" t="str">
-        <v>Chrome</v>
+        <v>http://customerportal.dev-ts.online</v>
       </c>
       <c r="N8" t="str">
-        <v>Windows</v>
+        <v>Chrome</v>
       </c>
       <c r="O8" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P8" t="str">
         <v>See spec: tests/createticket.spec.js  TC: TC-TICKET-001</v>
       </c>
-      <c r="P8" t="str">
+      <c r="Q8" t="str">
         <v>All Playwright assertions pass</v>
       </c>
-      <c r="Q8" t="str">
+      <c r="R8" t="str">
         <v>Error: expect(page).toHaveTitle(expected) failed Expected pattern: /Create Ticket/i Received string: "Sign In" Timeout: 5000ms Call log: - Expect "toHaveTitle" with timeout 5000ms 14 × unexpected value "Sign In"</v>
       </c>
-      <c r="R8" t="str">
-        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
-      </c>
       <c r="S8" t="str">
-        <v>CreateTicket</v>
-      </c>
-      <c r="T8" t="str">
-        <v>Auto</v>
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
         <v>26 Jun 2026</v>
       </c>
+      <c r="B9" t="str">
+        <v>CreateTicket</v>
+      </c>
       <c r="C9" t="str">
         <v>TC-TICKET-005</v>
       </c>
@@ -911,55 +915,55 @@
         <v>Positive</v>
       </c>
       <c r="F9" t="str">
-        <v>Low</v>
+        <v>Auto</v>
       </c>
       <c r="G9" t="str">
-        <v>FAIL</v>
+        <v>Low</v>
       </c>
       <c r="H9" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I9" t="str">
         <v>BUG-CREATETICKET-008</v>
       </c>
-      <c r="I9" t="str">
+      <c r="J9" t="str">
         <v>[FAIL] TC-TICKET-005 | All Ticket Type chips are visible</v>
       </c>
-      <c r="J9" t="str">
-        <v>Low</v>
-      </c>
       <c r="K9" t="str">
-        <v>P3</v>
+        <v>Low</v>
       </c>
       <c r="L9" t="str">
-        <v>http://customerportal.dev-ts.online</v>
+        <v>P3</v>
       </c>
       <c r="M9" t="str">
-        <v>Chrome</v>
+        <v>http://customerportal.dev-ts.online</v>
       </c>
       <c r="N9" t="str">
-        <v>Windows</v>
+        <v>Chrome</v>
       </c>
       <c r="O9" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P9" t="str">
         <v>See spec: tests/createticket.spec.js  TC: TC-TICKET-005</v>
       </c>
-      <c r="P9" t="str">
+      <c r="Q9" t="str">
         <v>All Playwright assertions pass</v>
       </c>
-      <c r="Q9" t="str">
+      <c r="R9" t="str">
         <v>Error: expect(locator).toBeVisible() failed Locator: locator('#typeChips .ct-type-chip').filter({ hasText: 'New' }).first() Expected: visible Timeout: 5000ms Error: element(s) not found Call log: - Expect "toBeVisible" with timeout 5000ms - waiting for locator('#typeChips .ct-type-chip').filter({ ha</v>
       </c>
-      <c r="R9" t="str">
-        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
-      </c>
       <c r="S9" t="str">
-        <v>CreateTicket</v>
-      </c>
-      <c r="T9" t="str">
-        <v>Auto</v>
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
         <v>26 Jun 2026</v>
       </c>
+      <c r="B10" t="str">
+        <v>CreateTicket</v>
+      </c>
       <c r="C10" t="str">
         <v>TC-DASH-003</v>
       </c>
@@ -970,55 +974,55 @@
         <v>Positive</v>
       </c>
       <c r="F10" t="str">
-        <v>Low</v>
+        <v>Auto</v>
       </c>
       <c r="G10" t="str">
-        <v>FAIL</v>
+        <v>Low</v>
       </c>
       <c r="H10" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I10" t="str">
         <v>BUG-CREATETICKET-009</v>
       </c>
-      <c r="I10" t="str">
+      <c r="J10" t="str">
         <v>[FAIL] TC-DASH-003 | OVERVIEW and ANALYTICS buttons visible</v>
       </c>
-      <c r="J10" t="str">
-        <v>Low</v>
-      </c>
       <c r="K10" t="str">
-        <v>P3</v>
+        <v>Low</v>
       </c>
       <c r="L10" t="str">
-        <v>http://customerportal.dev-ts.online</v>
+        <v>P3</v>
       </c>
       <c r="M10" t="str">
-        <v>Chrome</v>
+        <v>http://customerportal.dev-ts.online</v>
       </c>
       <c r="N10" t="str">
-        <v>Windows</v>
+        <v>Chrome</v>
       </c>
       <c r="O10" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P10" t="str">
         <v>See spec: tests/createticket.spec.js  TC: TC-DASH-003</v>
       </c>
-      <c r="P10" t="str">
+      <c r="Q10" t="str">
         <v>All Playwright assertions pass</v>
       </c>
-      <c r="Q10" t="str">
+      <c r="R10" t="str">
         <v>Error: expect(locator).toBeVisible() failed Locator: locator('#btnOverview') Expected: visible Timeout: 5000ms Error: element(s) not found Call log: - Expect "toBeVisible" with timeout 5000ms - waiting for locator('#btnOverview')</v>
       </c>
-      <c r="R10" t="str">
-        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
-      </c>
       <c r="S10" t="str">
-        <v>CreateTicket</v>
-      </c>
-      <c r="T10" t="str">
-        <v>Auto</v>
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
         <v>26 Jun 2026</v>
       </c>
+      <c r="B11" t="str">
+        <v>CreateTicket</v>
+      </c>
       <c r="C11" t="str">
         <v>TC-DASH-009</v>
       </c>
@@ -1029,55 +1033,55 @@
         <v>Positive</v>
       </c>
       <c r="F11" t="str">
-        <v>Low</v>
+        <v>Auto</v>
       </c>
       <c r="G11" t="str">
-        <v>FAIL</v>
+        <v>Low</v>
       </c>
       <c r="H11" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I11" t="str">
         <v>BUG-CREATETICKET-010</v>
       </c>
-      <c r="I11" t="str">
+      <c r="J11" t="str">
         <v>[FAIL] TC-DASH-009 | Active Tickets table with correct columns</v>
       </c>
-      <c r="J11" t="str">
-        <v>Low</v>
-      </c>
       <c r="K11" t="str">
-        <v>P3</v>
+        <v>Low</v>
       </c>
       <c r="L11" t="str">
-        <v>http://customerportal.dev-ts.online</v>
+        <v>P3</v>
       </c>
       <c r="M11" t="str">
-        <v>Chrome</v>
+        <v>http://customerportal.dev-ts.online</v>
       </c>
       <c r="N11" t="str">
-        <v>Windows</v>
+        <v>Chrome</v>
       </c>
       <c r="O11" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P11" t="str">
         <v>See spec: tests/createticket.spec.js  TC: TC-DASH-009</v>
       </c>
-      <c r="P11" t="str">
+      <c r="Q11" t="str">
         <v>All Playwright assertions pass</v>
       </c>
-      <c r="Q11" t="str">
+      <c r="R11" t="str">
         <v>Error: expect(locator).toBeVisible() failed Locator: locator('table').first() Expected: visible Timeout: 5000ms Error: element(s) not found Call log: - Expect "toBeVisible" with timeout 5000ms - waiting for locator('table').first()</v>
       </c>
-      <c r="R11" t="str">
-        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
-      </c>
       <c r="S11" t="str">
-        <v>CreateTicket</v>
-      </c>
-      <c r="T11" t="str">
-        <v>Auto</v>
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
         <v>26 Jun 2026</v>
       </c>
+      <c r="B12" t="str">
+        <v>CreateTicket</v>
+      </c>
       <c r="C12" t="str">
         <v>TC-DASH-013</v>
       </c>
@@ -1088,55 +1092,55 @@
         <v>Positive</v>
       </c>
       <c r="F12" t="str">
-        <v>Low</v>
+        <v>Auto</v>
       </c>
       <c r="G12" t="str">
-        <v>FAIL</v>
+        <v>Low</v>
       </c>
       <c r="H12" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I12" t="str">
         <v>BUG-CREATETICKET-011</v>
       </c>
-      <c r="I12" t="str">
+      <c r="J12" t="str">
         <v>[FAIL] TC-DASH-013 | Search box accepts input</v>
       </c>
-      <c r="J12" t="str">
-        <v>Low</v>
-      </c>
       <c r="K12" t="str">
-        <v>P3</v>
+        <v>Low</v>
       </c>
       <c r="L12" t="str">
-        <v>http://customerportal.dev-ts.online</v>
+        <v>P3</v>
       </c>
       <c r="M12" t="str">
-        <v>Chrome</v>
+        <v>http://customerportal.dev-ts.online</v>
       </c>
       <c r="N12" t="str">
-        <v>Windows</v>
+        <v>Chrome</v>
       </c>
       <c r="O12" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P12" t="str">
         <v>See spec: tests/createticket.spec.js  TC: TC-DASH-013</v>
       </c>
-      <c r="P12" t="str">
+      <c r="Q12" t="str">
         <v>All Playwright assertions pass</v>
       </c>
-      <c r="Q12" t="str">
+      <c r="R12" t="str">
         <v>Error: expect(locator).toBeVisible() failed Locator: locator('input[placeholder="Search"]').first() Expected: visible Timeout: 5000ms Error: element(s) not found Call log: - Expect "toBeVisible" with timeout 5000ms - waiting for locator('input[placeholder="Search"]').first()</v>
       </c>
-      <c r="R12" t="str">
-        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
-      </c>
       <c r="S12" t="str">
-        <v>CreateTicket</v>
-      </c>
-      <c r="T12" t="str">
-        <v>Auto</v>
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
         <v>26 Jun 2026</v>
       </c>
+      <c r="B13" t="str">
+        <v>CreateTicket</v>
+      </c>
       <c r="C13" t="str">
         <v>CreateTicket-passed-26 Jun 2026</v>
       </c>
@@ -1150,52 +1154,52 @@
         <v>Mixed</v>
       </c>
       <c r="G13" t="str">
+        <v>Mixed</v>
+      </c>
+      <c r="H13" t="str">
         <v>PASS</v>
       </c>
-      <c r="H13" t="str">
+      <c r="I13" t="str">
         <v>—</v>
       </c>
-      <c r="I13" t="str">
+      <c r="J13" t="str">
         <v>25/55 TCs passed</v>
-      </c>
-      <c r="J13" t="str">
-        <v>—</v>
       </c>
       <c r="K13" t="str">
         <v>—</v>
       </c>
       <c r="L13" t="str">
-        <v>http://customerportal.dev-ts.online</v>
+        <v>—</v>
       </c>
       <c r="M13" t="str">
-        <v>Chrome</v>
+        <v>http://customerportal.dev-ts.online</v>
       </c>
       <c r="N13" t="str">
-        <v>Windows</v>
+        <v>Chrome</v>
       </c>
       <c r="O13" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P13" t="str">
         <v>Playwright run: tests/createticket.spec.js</v>
       </c>
-      <c r="P13" t="str">
+      <c r="Q13" t="str">
         <v>Assertions pass</v>
       </c>
-      <c r="Q13" t="str">
+      <c r="R13" t="str">
         <v>25/55 PASS | 10 FAILs logged</v>
       </c>
-      <c r="R13" t="str">
-        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
-      </c>
       <c r="S13" t="str">
-        <v>CreateTicket</v>
-      </c>
-      <c r="T13" t="str">
-        <v>Mixed</v>
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
         <v>26 Jun 2026</v>
       </c>
+      <c r="B14" t="str">
+        <v>Dashboard</v>
+      </c>
       <c r="C14" t="str">
         <v>Dashboard-passed-26 Jun 2026</v>
       </c>
@@ -1209,52 +1213,52 @@
         <v>Mixed</v>
       </c>
       <c r="G14" t="str">
+        <v>Mixed</v>
+      </c>
+      <c r="H14" t="str">
         <v>PASS</v>
       </c>
-      <c r="H14" t="str">
+      <c r="I14" t="str">
         <v>—</v>
       </c>
-      <c r="I14" t="str">
+      <c r="J14" t="str">
         <v>25/55 TCs passed</v>
-      </c>
-      <c r="J14" t="str">
-        <v>—</v>
       </c>
       <c r="K14" t="str">
         <v>—</v>
       </c>
       <c r="L14" t="str">
-        <v>http://customerportal.dev-ts.online</v>
+        <v>—</v>
       </c>
       <c r="M14" t="str">
-        <v>Chrome</v>
+        <v>http://customerportal.dev-ts.online</v>
       </c>
       <c r="N14" t="str">
-        <v>Windows</v>
+        <v>Chrome</v>
       </c>
       <c r="O14" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P14" t="str">
         <v>Playwright run: tests/dashboard.spec.js</v>
       </c>
-      <c r="P14" t="str">
+      <c r="Q14" t="str">
         <v>Assertions pass</v>
       </c>
-      <c r="Q14" t="str">
+      <c r="R14" t="str">
         <v>25/55 PASS | 10 FAILs logged</v>
       </c>
-      <c r="R14" t="str">
+      <c r="S14" t="str">
         <v>Test Execution Report\Feature Reports\Dashboard.xlsx</v>
-      </c>
-      <c r="S14" t="str">
-        <v>Dashboard</v>
-      </c>
-      <c r="T14" t="str">
-        <v>Mixed</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
         <v>26 Jun 2026</v>
       </c>
+      <c r="B15" t="str">
+        <v>Login</v>
+      </c>
       <c r="C15" t="str">
         <v>Login-passed-26 Jun 2026</v>
       </c>
@@ -1268,51 +1272,1228 @@
         <v>Mixed</v>
       </c>
       <c r="G15" t="str">
+        <v>Mixed</v>
+      </c>
+      <c r="H15" t="str">
         <v>PASS</v>
       </c>
-      <c r="H15" t="str">
+      <c r="I15" t="str">
         <v>—</v>
       </c>
-      <c r="I15" t="str">
+      <c r="J15" t="str">
         <v>25/55 TCs passed</v>
-      </c>
-      <c r="J15" t="str">
-        <v>—</v>
       </c>
       <c r="K15" t="str">
         <v>—</v>
       </c>
       <c r="L15" t="str">
-        <v>http://customerportal.dev-ts.online</v>
+        <v>—</v>
       </c>
       <c r="M15" t="str">
-        <v>Chrome</v>
+        <v>http://customerportal.dev-ts.online</v>
       </c>
       <c r="N15" t="str">
-        <v>Windows</v>
+        <v>Chrome</v>
       </c>
       <c r="O15" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P15" t="str">
         <v>Playwright run: tests/login.spec.js</v>
       </c>
-      <c r="P15" t="str">
+      <c r="Q15" t="str">
         <v>Assertions pass</v>
       </c>
-      <c r="Q15" t="str">
+      <c r="R15" t="str">
         <v>25/55 PASS | 10 FAILs logged</v>
       </c>
-      <c r="R15" t="str">
+      <c r="S15" t="str">
         <v>Test Execution Report\Feature Reports\Login.xlsx</v>
       </c>
-      <c r="S15" t="str">
-        <v>Login</v>
-      </c>
-      <c r="T15" t="str">
-        <v>Mixed</v>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="B16" t="str">
+        <v>CreateTicket</v>
+      </c>
+      <c r="C16" t="str">
+        <v>TC-TICKET-002</v>
+      </c>
+      <c r="D16" t="str">
+        <v>TC-TICKET-002 | Submit ticket with all required fields filled</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F16" t="str">
+        <v>API</v>
+      </c>
+      <c r="G16" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H16" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I16" t="str">
+        <v>BUG-CREATETICKET-012</v>
+      </c>
+      <c r="J16" t="str">
+        <v>[FAIL] TC-TICKET-002 | Submit ticket with all required fields filled</v>
+      </c>
+      <c r="K16" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L16" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M16" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N16" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O16" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P16" t="str">
+        <v>See spec: tests/createticket.spec.js  TC: TC-TICKET-002</v>
+      </c>
+      <c r="Q16" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R16" t="str">
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('input[placeholder="Select Project..."]')</v>
+      </c>
+      <c r="S16" t="str">
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="B17" t="str">
+        <v>CreateTicket</v>
+      </c>
+      <c r="C17" t="str">
+        <v>TC-TICKET-003</v>
+      </c>
+      <c r="D17" t="str">
+        <v>TC-TICKET-003 | Project dropdown shows all available projects</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F17" t="str">
+        <v>API</v>
+      </c>
+      <c r="G17" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H17" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I17" t="str">
+        <v>BUG-CREATETICKET-013</v>
+      </c>
+      <c r="J17" t="str">
+        <v>[FAIL] TC-TICKET-003 | Project dropdown shows all available projects</v>
+      </c>
+      <c r="K17" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L17" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M17" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N17" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O17" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P17" t="str">
+        <v>See spec: tests/createticket.spec.js  TC: TC-TICKET-003</v>
+      </c>
+      <c r="Q17" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R17" t="str">
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('input[placeholder="Select Project..."]')</v>
+      </c>
+      <c r="S17" t="str">
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="B18" t="str">
+        <v>CreateTicket</v>
+      </c>
+      <c r="C18" t="str">
+        <v>TC-TICKET-004</v>
+      </c>
+      <c r="D18" t="str">
+        <v>TC-TICKET-004 | Selecting project unlocks Platform dropdown</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F18" t="str">
+        <v>API</v>
+      </c>
+      <c r="G18" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H18" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I18" t="str">
+        <v>BUG-CREATETICKET-014</v>
+      </c>
+      <c r="J18" t="str">
+        <v>[FAIL] TC-TICKET-004 | Selecting project unlocks Platform dropdown</v>
+      </c>
+      <c r="K18" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L18" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M18" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N18" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O18" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P18" t="str">
+        <v>See spec: tests/createticket.spec.js  TC: TC-TICKET-004</v>
+      </c>
+      <c r="Q18" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R18" t="str">
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('input[placeholder="Select Project..."]')</v>
+      </c>
+      <c r="S18" t="str">
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="B19" t="str">
+        <v>CreateTicket</v>
+      </c>
+      <c r="C19" t="str">
+        <v>TC-TICKET-006</v>
+      </c>
+      <c r="D19" t="str">
+        <v>TC-TICKET-006 | Description character counter updates on input</v>
+      </c>
+      <c r="E19" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F19" t="str">
+        <v>API</v>
+      </c>
+      <c r="G19" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H19" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I19" t="str">
+        <v>BUG-CREATETICKET-015</v>
+      </c>
+      <c r="J19" t="str">
+        <v>[FAIL] TC-TICKET-006 | Description character counter updates on input</v>
+      </c>
+      <c r="K19" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L19" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M19" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N19" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O19" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P19" t="str">
+        <v>See spec: tests/createticket.spec.js  TC: TC-TICKET-006</v>
+      </c>
+      <c r="Q19" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R19" t="str">
+        <v>TimeoutError: locator.fill: Timeout 15000ms exceeded. Call log: - waiting for locator('#txtDescription')</v>
+      </c>
+      <c r="S19" t="str">
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="B20" t="str">
+        <v>CreateTicket</v>
+      </c>
+      <c r="C20" t="str">
+        <v>TC-TICKET-007</v>
+      </c>
+      <c r="D20" t="str">
+        <v>TC-TICKET-007 | Reset button clears all filled fields</v>
+      </c>
+      <c r="E20" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F20" t="str">
+        <v>API</v>
+      </c>
+      <c r="G20" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H20" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I20" t="str">
+        <v>BUG-CREATETICKET-016</v>
+      </c>
+      <c r="J20" t="str">
+        <v>[FAIL] TC-TICKET-007 | Reset button clears all filled fields</v>
+      </c>
+      <c r="K20" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L20" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M20" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N20" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O20" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P20" t="str">
+        <v>See spec: tests/createticket.spec.js  TC: TC-TICKET-007</v>
+      </c>
+      <c r="Q20" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R20" t="str">
+        <v>TimeoutError: locator.fill: Timeout 15000ms exceeded. Call log: - waiting for locator('#txtPageName')</v>
+      </c>
+      <c r="S20" t="str">
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="B21" t="str">
+        <v>CreateTicket</v>
+      </c>
+      <c r="C21" t="str">
+        <v>TC-TICKET-008</v>
+      </c>
+      <c r="D21" t="str">
+        <v>TC-TICKET-008 | Page/Screen Name field is optional</v>
+      </c>
+      <c r="E21" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F21" t="str">
+        <v>API</v>
+      </c>
+      <c r="G21" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H21" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I21" t="str">
+        <v>BUG-CREATETICKET-017</v>
+      </c>
+      <c r="J21" t="str">
+        <v>[FAIL] TC-TICKET-008 | Page/Screen Name field is optional</v>
+      </c>
+      <c r="K21" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L21" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M21" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N21" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O21" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P21" t="str">
+        <v>See spec: tests/createticket.spec.js  TC: TC-TICKET-008</v>
+      </c>
+      <c r="Q21" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R21" t="str">
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('input[placeholder="Select Project..."]')</v>
+      </c>
+      <c r="S21" t="str">
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="B22" t="str">
+        <v>CreateTicket</v>
+      </c>
+      <c r="C22" t="str">
+        <v>TC-TICKET-009</v>
+      </c>
+      <c r="D22" t="str">
+        <v>TC-TICKET-009 | Submit with no fields filled shows validation popup</v>
+      </c>
+      <c r="E22" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F22" t="str">
+        <v>API</v>
+      </c>
+      <c r="G22" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H22" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I22" t="str">
+        <v>BUG-CREATETICKET-018</v>
+      </c>
+      <c r="J22" t="str">
+        <v>[FAIL] TC-TICKET-009 | Submit with no fields filled shows validation popup</v>
+      </c>
+      <c r="K22" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L22" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M22" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N22" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O22" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P22" t="str">
+        <v>See spec: tests/createticket.spec.js  TC: TC-TICKET-009</v>
+      </c>
+      <c r="Q22" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R22" t="str">
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for getByRole('button', { name: /submit ticket/i })</v>
+      </c>
+      <c r="S22" t="str">
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="B23" t="str">
+        <v>CreateTicket</v>
+      </c>
+      <c r="C23" t="str">
+        <v>TC-TICKET-010</v>
+      </c>
+      <c r="D23" t="str">
+        <v>TC-TICKET-010 | Submit without Project shows Missing Information</v>
+      </c>
+      <c r="E23" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F23" t="str">
+        <v>API</v>
+      </c>
+      <c r="G23" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H23" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I23" t="str">
+        <v>BUG-CREATETICKET-019</v>
+      </c>
+      <c r="J23" t="str">
+        <v>[FAIL] TC-TICKET-010 | Submit without Project shows Missing Information</v>
+      </c>
+      <c r="K23" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L23" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M23" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N23" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O23" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P23" t="str">
+        <v>See spec: tests/createticket.spec.js  TC: TC-TICKET-010</v>
+      </c>
+      <c r="Q23" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R23" t="str">
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('input[placeholder="Select Type..."]')</v>
+      </c>
+      <c r="S23" t="str">
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="B24" t="str">
+        <v>CreateTicket</v>
+      </c>
+      <c r="C24" t="str">
+        <v>TC-TICKET-011</v>
+      </c>
+      <c r="D24" t="str">
+        <v>TC-TICKET-011 | Submit without Ticket Type shows validation error</v>
+      </c>
+      <c r="E24" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F24" t="str">
+        <v>API</v>
+      </c>
+      <c r="G24" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H24" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I24" t="str">
+        <v>BUG-CREATETICKET-020</v>
+      </c>
+      <c r="J24" t="str">
+        <v>[FAIL] TC-TICKET-011 | Submit without Ticket Type shows validation error</v>
+      </c>
+      <c r="K24" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L24" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M24" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N24" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O24" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P24" t="str">
+        <v>See spec: tests/createticket.spec.js  TC: TC-TICKET-011</v>
+      </c>
+      <c r="Q24" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R24" t="str">
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('input[placeholder="Select Project..."]')</v>
+      </c>
+      <c r="S24" t="str">
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="B25" t="str">
+        <v>CreateTicket</v>
+      </c>
+      <c r="C25" t="str">
+        <v>TC-TICKET-012</v>
+      </c>
+      <c r="D25" t="str">
+        <v>TC-TICKET-012 | Submit without Description shows validation error</v>
+      </c>
+      <c r="E25" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F25" t="str">
+        <v>API</v>
+      </c>
+      <c r="G25" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H25" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I25" t="str">
+        <v>BUG-CREATETICKET-021</v>
+      </c>
+      <c r="J25" t="str">
+        <v>[FAIL] TC-TICKET-012 | Submit without Description shows validation error</v>
+      </c>
+      <c r="K25" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L25" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M25" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N25" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O25" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P25" t="str">
+        <v>See spec: tests/createticket.spec.js  TC: TC-TICKET-012</v>
+      </c>
+      <c r="Q25" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R25" t="str">
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('input[placeholder="Select Project..."]')</v>
+      </c>
+      <c r="S25" t="str">
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="B26" t="str">
+        <v>CreateTicket</v>
+      </c>
+      <c r="C26" t="str">
+        <v>TC-TICKET-013</v>
+      </c>
+      <c r="D26" t="str">
+        <v>TC-TICKET-013 | Submit without Platform shows validation error</v>
+      </c>
+      <c r="E26" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F26" t="str">
+        <v>API</v>
+      </c>
+      <c r="G26" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H26" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I26" t="str">
+        <v>BUG-CREATETICKET-022</v>
+      </c>
+      <c r="J26" t="str">
+        <v>[FAIL] TC-TICKET-013 | Submit without Platform shows validation error</v>
+      </c>
+      <c r="K26" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L26" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M26" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N26" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O26" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P26" t="str">
+        <v>See spec: tests/createticket.spec.js  TC: TC-TICKET-013</v>
+      </c>
+      <c r="Q26" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R26" t="str">
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('input[placeholder="Select Project..."]')</v>
+      </c>
+      <c r="S26" t="str">
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="B27" t="str">
+        <v>CreateTicket</v>
+      </c>
+      <c r="C27" t="str">
+        <v>TC-TICKET-014</v>
+      </c>
+      <c r="D27" t="str">
+        <v>TC-TICKET-014 | Description with exactly 14 chars fails validation</v>
+      </c>
+      <c r="E27" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F27" t="str">
+        <v>API</v>
+      </c>
+      <c r="G27" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H27" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I27" t="str">
+        <v>BUG-CREATETICKET-023</v>
+      </c>
+      <c r="J27" t="str">
+        <v>[FAIL] TC-TICKET-014 | Description with exactly 14 chars fails validation</v>
+      </c>
+      <c r="K27" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L27" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M27" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N27" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O27" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P27" t="str">
+        <v>See spec: tests/createticket.spec.js  TC: TC-TICKET-014</v>
+      </c>
+      <c r="Q27" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R27" t="str">
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('input[placeholder="Select Project..."]')</v>
+      </c>
+      <c r="S27" t="str">
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="B28" t="str">
+        <v>CreateTicket</v>
+      </c>
+      <c r="C28" t="str">
+        <v>TC-TICKET-015</v>
+      </c>
+      <c r="D28" t="str">
+        <v>TC-TICKET-015 | Description with exactly 15 chars passes validation</v>
+      </c>
+      <c r="E28" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F28" t="str">
+        <v>API</v>
+      </c>
+      <c r="G28" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H28" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I28" t="str">
+        <v>BUG-CREATETICKET-024</v>
+      </c>
+      <c r="J28" t="str">
+        <v>[FAIL] TC-TICKET-015 | Description with exactly 15 chars passes validation</v>
+      </c>
+      <c r="K28" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L28" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M28" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N28" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O28" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P28" t="str">
+        <v>See spec: tests/createticket.spec.js  TC: TC-TICKET-015</v>
+      </c>
+      <c r="Q28" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R28" t="str">
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('input[placeholder="Select Project..."]')</v>
+      </c>
+      <c r="S28" t="str">
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="B29" t="str">
+        <v>CreateTicket</v>
+      </c>
+      <c r="C29" t="str">
+        <v>TC-TICKET-016</v>
+      </c>
+      <c r="D29" t="str">
+        <v>TC-TICKET-016 | Description at 2000 chars (max) is accepted</v>
+      </c>
+      <c r="E29" t="str">
+        <v>Boundary</v>
+      </c>
+      <c r="F29" t="str">
+        <v>API</v>
+      </c>
+      <c r="G29" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="H29" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I29" t="str">
+        <v>BUG-CREATETICKET-025</v>
+      </c>
+      <c r="J29" t="str">
+        <v>[FAIL] TC-TICKET-016 | Description at 2000 chars (max) is accepted</v>
+      </c>
+      <c r="K29" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="L29" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M29" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N29" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O29" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P29" t="str">
+        <v>See spec: tests/createticket.spec.js  TC: TC-TICKET-016</v>
+      </c>
+      <c r="Q29" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R29" t="str">
+        <v>TimeoutError: locator.fill: Timeout 15000ms exceeded. Call log: - waiting for locator('#txtDescription')</v>
+      </c>
+      <c r="S29" t="str">
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="B30" t="str">
+        <v>CreateTicket</v>
+      </c>
+      <c r="C30" t="str">
+        <v>TC-TICKET-017</v>
+      </c>
+      <c r="D30" t="str">
+        <v>TC-TICKET-017 | Platform chips show all expected options after project selected</v>
+      </c>
+      <c r="E30" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F30" t="str">
+        <v>API</v>
+      </c>
+      <c r="G30" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H30" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I30" t="str">
+        <v>BUG-CREATETICKET-026</v>
+      </c>
+      <c r="J30" t="str">
+        <v>[FAIL] TC-TICKET-017 | Platform chips show all expected options after project selected</v>
+      </c>
+      <c r="K30" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L30" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M30" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N30" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O30" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P30" t="str">
+        <v>See spec: tests/createticket.spec.js  TC: TC-TICKET-017</v>
+      </c>
+      <c r="Q30" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R30" t="str">
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('input[placeholder="Select Project..."]')</v>
+      </c>
+      <c r="S30" t="str">
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="B31" t="str">
+        <v>CreateTicket</v>
+      </c>
+      <c r="C31" t="str">
+        <v>TC-TICKET-018</v>
+      </c>
+      <c r="D31" t="str">
+        <v>TC-TICKET-018 | SQL injection in description is handled safely</v>
+      </c>
+      <c r="E31" t="str">
+        <v>Security</v>
+      </c>
+      <c r="F31" t="str">
+        <v>API</v>
+      </c>
+      <c r="G31" t="str">
+        <v>High</v>
+      </c>
+      <c r="H31" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I31" t="str">
+        <v>BUG-CREATETICKET-027</v>
+      </c>
+      <c r="J31" t="str">
+        <v>[FAIL] TC-TICKET-018 | SQL injection in description is handled safely</v>
+      </c>
+      <c r="K31" t="str">
+        <v>High</v>
+      </c>
+      <c r="L31" t="str">
+        <v>P2</v>
+      </c>
+      <c r="M31" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N31" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O31" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P31" t="str">
+        <v>See spec: tests/createticket.spec.js  TC: TC-TICKET-018</v>
+      </c>
+      <c r="Q31" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R31" t="str">
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('input[placeholder="Select Project..."]')</v>
+      </c>
+      <c r="S31" t="str">
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="B32" t="str">
+        <v>CreateTicket</v>
+      </c>
+      <c r="C32" t="str">
+        <v>TC-TICKET-019</v>
+      </c>
+      <c r="D32" t="str">
+        <v>TC-TICKET-019 | XSS payload in description is handled safely</v>
+      </c>
+      <c r="E32" t="str">
+        <v>Security</v>
+      </c>
+      <c r="F32" t="str">
+        <v>API</v>
+      </c>
+      <c r="G32" t="str">
+        <v>High</v>
+      </c>
+      <c r="H32" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I32" t="str">
+        <v>BUG-CREATETICKET-028</v>
+      </c>
+      <c r="J32" t="str">
+        <v>[FAIL] TC-TICKET-019 | XSS payload in description is handled safely</v>
+      </c>
+      <c r="K32" t="str">
+        <v>High</v>
+      </c>
+      <c r="L32" t="str">
+        <v>P2</v>
+      </c>
+      <c r="M32" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N32" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O32" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P32" t="str">
+        <v>See spec: tests/createticket.spec.js  TC: TC-TICKET-019</v>
+      </c>
+      <c r="Q32" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R32" t="str">
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('input[placeholder="Select Project..."]')</v>
+      </c>
+      <c r="S32" t="str">
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="B33" t="str">
+        <v>CreateTicket</v>
+      </c>
+      <c r="C33" t="str">
+        <v>TC-DASH-006</v>
+      </c>
+      <c r="D33" t="str">
+        <v>TC-DASH-006 | Date range filter applies correctly</v>
+      </c>
+      <c r="E33" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F33" t="str">
+        <v>API</v>
+      </c>
+      <c r="G33" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H33" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I33" t="str">
+        <v>BUG-CREATETICKET-029</v>
+      </c>
+      <c r="J33" t="str">
+        <v>[FAIL] TC-DASH-006 | Date range filter applies correctly</v>
+      </c>
+      <c r="K33" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L33" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M33" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N33" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O33" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P33" t="str">
+        <v>See spec: tests/createticket.spec.js  TC: TC-DASH-006</v>
+      </c>
+      <c r="Q33" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R33" t="str">
+        <v>TimeoutError: locator.fill: Timeout 15000ms exceeded. Call log: - waiting for locator('#dr_from') - locator resolved to &lt;input type="date" id="dr_from" max="2026-06-26" class="w-full text-[0.75rem] py-1.5 px-2 border border-gray-200 rounded mb-2 dark:bg-[#1a1a2e] dark:border-[#2b2b40] dark:text-gray</v>
+      </c>
+      <c r="S33" t="str">
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="B34" t="str">
+        <v>CreateTicket</v>
+      </c>
+      <c r="C34" t="str">
+        <v>TC-DASH-007</v>
+      </c>
+      <c r="D34" t="str">
+        <v>TC-DASH-007 | Reset button clears date filter</v>
+      </c>
+      <c r="E34" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F34" t="str">
+        <v>API</v>
+      </c>
+      <c r="G34" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H34" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I34" t="str">
+        <v>BUG-CREATETICKET-030</v>
+      </c>
+      <c r="J34" t="str">
+        <v>[FAIL] TC-DASH-007 | Reset button clears date filter</v>
+      </c>
+      <c r="K34" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L34" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M34" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N34" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O34" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P34" t="str">
+        <v>See spec: tests/createticket.spec.js  TC: TC-DASH-007</v>
+      </c>
+      <c r="Q34" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R34" t="str">
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('#dr_apply') - locator resolved to &lt;button id="dr_apply" class="w-full text-[0.75rem] font-bold text-white bg-blue-600 hover:bg-blue-700 rounded py-1.5 transition-colors"&gt;Apply Range&lt;/button&gt; - attempting click ac</v>
+      </c>
+      <c r="S34" t="str">
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="B35" t="str">
+        <v>CreateTicket</v>
+      </c>
+      <c r="C35" t="str">
+        <v>TC-DASH-008</v>
+      </c>
+      <c r="D35" t="str">
+        <v>TC-DASH-008 | Invalid date range To &lt; From handled gracefully</v>
+      </c>
+      <c r="E35" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F35" t="str">
+        <v>API</v>
+      </c>
+      <c r="G35" t="str">
+        <v>High</v>
+      </c>
+      <c r="H35" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I35" t="str">
+        <v>BUG-CREATETICKET-031</v>
+      </c>
+      <c r="J35" t="str">
+        <v>[FAIL] TC-DASH-008 | Invalid date range To &lt; From handled gracefully</v>
+      </c>
+      <c r="K35" t="str">
+        <v>High</v>
+      </c>
+      <c r="L35" t="str">
+        <v>P2</v>
+      </c>
+      <c r="M35" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N35" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O35" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P35" t="str">
+        <v>See spec: tests/createticket.spec.js  TC: TC-DASH-008</v>
+      </c>
+      <c r="Q35" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R35" t="str">
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('#dr_apply') - locator resolved to &lt;button id="dr_apply" class="w-full text-[0.75rem] font-bold text-white bg-blue-600 hover:bg-blue-700 rounded py-1.5 transition-colors"&gt;Apply Range&lt;/button&gt; - attempting click ac</v>
+      </c>
+      <c r="S35" t="str">
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:T15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:T35"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
test: Login 20/20 PASS - Playwright auto-save report - fix CI scope detection
</commit_message>
<xml_diff>
--- a/Test Execution Report/Daily Reports/BugReport_26-Jun-2026.xlsx
+++ b/Test Execution Report/Daily Reports/BugReport_26-Jun-2026.xlsx
@@ -408,7 +408,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T35"/>
+  <dimension ref="A1:T36"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -2491,9 +2491,68 @@
         <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Login</v>
+      </c>
+      <c r="C36" t="str">
+        <v>TC-LOGIN-001-summary</v>
+      </c>
+      <c r="D36" t="str">
+        <v>All 20 TCs — Login module (TC-LOGIN-001 → TC-LOGIN-020)</v>
+      </c>
+      <c r="E36" t="str">
+        <v>All types</v>
+      </c>
+      <c r="F36" t="str">
+        <v>Unit / API / Auto</v>
+      </c>
+      <c r="G36" t="str">
+        <v>Critical–Low</v>
+      </c>
+      <c r="H36" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="I36" t="str">
+        <v>—</v>
+      </c>
+      <c r="J36" t="str">
+        <v>No bugs — 20/20 TCs passed</v>
+      </c>
+      <c r="K36" t="str">
+        <v>—</v>
+      </c>
+      <c r="L36" t="str">
+        <v>—</v>
+      </c>
+      <c r="M36" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N36" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O36" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P36" t="str">
+        <v>20 TCs via Playwright (tests/login.spec.js)</v>
+      </c>
+      <c r="Q36" t="str">
+        <v>All 20 TCs pass</v>
+      </c>
+      <c r="R36" t="str">
+        <v>20/20 PASS ✓  Pass Rate: 100%</v>
+      </c>
+      <c r="S36" t="str">
+        <v>Test Execution Report\Feature Reports\Login.xlsx</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:T35"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:T36"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
CI Reports [2026-06-26 14:20]: All — Excel reports updated
</commit_message>
<xml_diff>
--- a/Test Execution Report/Daily Reports/BugReport_26-Jun-2026.xlsx
+++ b/Test Execution Report/Daily Reports/BugReport_26-Jun-2026.xlsx
@@ -408,7 +408,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T36"/>
+  <dimension ref="A1:T39"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -2550,9 +2550,186 @@
         <v>Test Execution Report\Feature Reports\Login.xlsx</v>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="B37" t="str">
+        <v>CreateTicket</v>
+      </c>
+      <c r="C37" t="str">
+        <v>CreateTicket-summary</v>
+      </c>
+      <c r="D37" t="str">
+        <v>All 0 TCs — CreateTicket module (TC-CREATETICKET-001 → )</v>
+      </c>
+      <c r="E37" t="str">
+        <v>All types</v>
+      </c>
+      <c r="F37" t="str">
+        <v>Unit / API / Auto</v>
+      </c>
+      <c r="G37" t="str">
+        <v>Critical–Low</v>
+      </c>
+      <c r="H37" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="I37" t="str">
+        <v>—</v>
+      </c>
+      <c r="J37" t="str">
+        <v>No bugs — 0/0 TCs passed</v>
+      </c>
+      <c r="K37" t="str">
+        <v>—</v>
+      </c>
+      <c r="L37" t="str">
+        <v>—</v>
+      </c>
+      <c r="M37" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N37" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O37" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P37" t="str">
+        <v>0 TCs via Playwright (tests/createticket.spec.js)</v>
+      </c>
+      <c r="Q37" t="str">
+        <v>All 0 TCs pass</v>
+      </c>
+      <c r="R37" t="str">
+        <v>0/0 PASS ✓  Pass Rate: 100%</v>
+      </c>
+      <c r="S37" t="str">
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Dashboard</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Dashboard-summary</v>
+      </c>
+      <c r="D38" t="str">
+        <v>All 0 TCs — Dashboard module (TC-DASHBOARD-001 → )</v>
+      </c>
+      <c r="E38" t="str">
+        <v>All types</v>
+      </c>
+      <c r="F38" t="str">
+        <v>Unit / API / Auto</v>
+      </c>
+      <c r="G38" t="str">
+        <v>Critical–Low</v>
+      </c>
+      <c r="H38" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="I38" t="str">
+        <v>—</v>
+      </c>
+      <c r="J38" t="str">
+        <v>No bugs — 0/0 TCs passed</v>
+      </c>
+      <c r="K38" t="str">
+        <v>—</v>
+      </c>
+      <c r="L38" t="str">
+        <v>—</v>
+      </c>
+      <c r="M38" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N38" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O38" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P38" t="str">
+        <v>0 TCs via Playwright (tests/dashboard.spec.js)</v>
+      </c>
+      <c r="Q38" t="str">
+        <v>All 0 TCs pass</v>
+      </c>
+      <c r="R38" t="str">
+        <v>0/0 PASS ✓  Pass Rate: 100%</v>
+      </c>
+      <c r="S38" t="str">
+        <v>Test Execution Report\Feature Reports\Dashboard.xlsx</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Login</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Login-summary</v>
+      </c>
+      <c r="D39" t="str">
+        <v>All 0 TCs — Login module (TC-LOGIN-001 → )</v>
+      </c>
+      <c r="E39" t="str">
+        <v>All types</v>
+      </c>
+      <c r="F39" t="str">
+        <v>Unit / API / Auto</v>
+      </c>
+      <c r="G39" t="str">
+        <v>Critical–Low</v>
+      </c>
+      <c r="H39" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="I39" t="str">
+        <v>—</v>
+      </c>
+      <c r="J39" t="str">
+        <v>No bugs — 0/0 TCs passed</v>
+      </c>
+      <c r="K39" t="str">
+        <v>—</v>
+      </c>
+      <c r="L39" t="str">
+        <v>—</v>
+      </c>
+      <c r="M39" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N39" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O39" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P39" t="str">
+        <v>0 TCs via Playwright (tests/login.spec.js)</v>
+      </c>
+      <c r="Q39" t="str">
+        <v>All 0 TCs pass</v>
+      </c>
+      <c r="R39" t="str">
+        <v>0/0 PASS ✓  Pass Rate: 100%</v>
+      </c>
+      <c r="S39" t="str">
+        <v>Test Execution Report\Feature Reports\Login.xlsx</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:T36"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:T39"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
CI Reports [2026-06-26 14:53]: All — Excel reports updated
</commit_message>
<xml_diff>
--- a/Test Execution Report/Daily Reports/BugReport_26-Jun-2026.xlsx
+++ b/Test Execution Report/Daily Reports/BugReport_26-Jun-2026.xlsx
@@ -408,7 +408,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T39"/>
+  <dimension ref="A1:T41"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -2727,9 +2727,127 @@
         <v>Test Execution Report\Feature Reports\Login.xlsx</v>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="B40" t="str">
+        <v>CreateTicket</v>
+      </c>
+      <c r="C40" t="str">
+        <v>TC-TICKET-021</v>
+      </c>
+      <c r="D40" t="str">
+        <v>TC-TICKET-021 | Unauthenticated access redirected to login</v>
+      </c>
+      <c r="E40" t="str">
+        <v>Security</v>
+      </c>
+      <c r="F40" t="str">
+        <v>Auto</v>
+      </c>
+      <c r="G40" t="str">
+        <v>High</v>
+      </c>
+      <c r="H40" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I40" t="str">
+        <v>BUG-CREATETICKET-032</v>
+      </c>
+      <c r="J40" t="str">
+        <v>[FAIL] TC-TICKET-021 | Unauthenticated access redirected to login</v>
+      </c>
+      <c r="K40" t="str">
+        <v>High</v>
+      </c>
+      <c r="L40" t="str">
+        <v>P2</v>
+      </c>
+      <c r="M40" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N40" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O40" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P40" t="str">
+        <v>See spec: tests/createticket.spec.js  TC: TC-TICKET-021</v>
+      </c>
+      <c r="Q40" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R40" t="str">
+        <v>Error: expect(page).toHaveURL(expected) failed Expected pattern: /Login|Account/i Received string: "http://customerportal.dev-ts.online/Ticket/Create" Timeout: 5000ms Call log: - Expect "toHaveURL" with timeout 5000ms 14 × unexpected value "http://customerportal.dev-ts.online/Ticket/Create"</v>
+      </c>
+      <c r="S40" t="str">
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>26 Jun 2026</v>
+      </c>
+      <c r="B41" t="str">
+        <v>CreateTicket</v>
+      </c>
+      <c r="C41" t="str">
+        <v>TC-LOGIN-016</v>
+      </c>
+      <c r="D41" t="str">
+        <v>TC-LOGIN-016 | SQL injection in username handled safely</v>
+      </c>
+      <c r="E41" t="str">
+        <v>Security</v>
+      </c>
+      <c r="F41" t="str">
+        <v>API</v>
+      </c>
+      <c r="G41" t="str">
+        <v>High</v>
+      </c>
+      <c r="H41" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I41" t="str">
+        <v>BUG-CREATETICKET-033</v>
+      </c>
+      <c r="J41" t="str">
+        <v>[FAIL] TC-LOGIN-016 | SQL injection in username handled safely</v>
+      </c>
+      <c r="K41" t="str">
+        <v>High</v>
+      </c>
+      <c r="L41" t="str">
+        <v>P2</v>
+      </c>
+      <c r="M41" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N41" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O41" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P41" t="str">
+        <v>See spec: tests/createticket.spec.js  TC: TC-LOGIN-016</v>
+      </c>
+      <c r="Q41" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R41" t="str">
+        <v>Error: expect(page).toHaveURL(expected) failed Expected pattern: /Login/ Received string: "" Timeout: 5000ms Call log: - Expect "toHaveURL" with timeout 5000ms - waiting for navigation to finish...</v>
+      </c>
+      <c r="S41" t="str">
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:T39"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:T41"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>